<commit_message>
fix export phôi tấm HRC2
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/HRC2_BBSL_PhoiTam.xlsx
+++ b/dataproduct.api/wwwroot/templates/HRC2_BBSL_PhoiTam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\BIEUMAU_SANXUAT\Source\dataproduct.BE\dataproduct.api\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E1C176-3AE1-4FF9-9E11-B0727BF1ECDD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF4B3435-5DF9-4F20-95A9-D6ECF9639DD7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="11805" xr2:uid="{8D26054B-D371-44B9-99F0-3A3B1380D846}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Máy đúc</t>
   </si>
@@ -63,36 +63,10 @@
     <t>TT PKH</t>
   </si>
   <si>
-    <t xml:space="preserve">        BIÊN BẢN GIAO NHẬN PHÔI TẤM</t>
-  </si>
-  <si>
-    <t>BM.40/QT.05.10</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="12"/>
-        <color indexed="8"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>Ngày hiệu lực:</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color indexed="8"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> 10/10/2025 </t>
-    </r>
-  </si>
-  <si>
-    <t>Lần sửa đổi: 02</t>
+    <t xml:space="preserve">   CHI TIẾT SẢN LƯỢNG PHÔI TẤM</t>
+  </si>
+  <si>
+    <t>OrderID</t>
   </si>
 </sst>
 </file>
@@ -582,92 +556,90 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FE70C8B-98CB-4803-B542-3EE340B9292E}">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.28515625" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="30.140625" customWidth="1"/>
-    <col min="7" max="7" width="19.140625" customWidth="1"/>
-    <col min="8" max="8" width="17.85546875" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" customWidth="1"/>
-    <col min="11" max="11" width="15.7109375" customWidth="1"/>
-    <col min="12" max="12" width="16.5703125" customWidth="1"/>
-    <col min="13" max="13" width="12.7109375" customWidth="1"/>
+    <col min="3" max="4" width="19.140625" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" customWidth="1"/>
+    <col min="7" max="7" width="30.140625" customWidth="1"/>
+    <col min="8" max="8" width="19.140625" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" customWidth="1"/>
+    <col min="10" max="10" width="13.140625" customWidth="1"/>
+    <col min="11" max="11" width="14.5703125" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" customWidth="1"/>
+    <col min="13" max="13" width="16.5703125" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="2"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="2"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="M2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="1"/>
     </row>
-    <row r="3" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="1"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="2"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
-      <c r="L3" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="M3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="1"/>
     </row>
-    <row r="4" spans="1:13" ht="73.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" ht="73.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="2"/>
       <c r="F4" s="6"/>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="6"/>
+      <c r="H4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="6"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
       <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
     </row>
-    <row r="5" spans="1:13" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>2</v>
       </c>
@@ -678,33 +650,36 @@
         <v>4</v>
       </c>
       <c r="D5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="I5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="J5" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="K5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="L5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="9" t="s">
+      <c r="M5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
thêm bảng check slab theo user
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/HRC2_BBSL_PhoiTam.xlsx
+++ b/dataproduct.api/wwwroot/templates/HRC2_BBSL_PhoiTam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\BIEUMAU_SANXUAT\Source\dataproduct.BE\dataproduct.api\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF4B3435-5DF9-4F20-95A9-D6ECF9639DD7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{493432AD-E8B0-4D75-BE7C-8FAC14464C5B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="11805" xr2:uid="{8D26054B-D371-44B9-99F0-3A3B1380D846}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Máy đúc</t>
   </si>
@@ -36,9 +36,6 @@
     <t>STT</t>
   </si>
   <si>
-    <t>Ca SX</t>
-  </si>
-  <si>
     <t>ID Slab</t>
   </si>
   <si>
@@ -67,6 +64,12 @@
   </si>
   <si>
     <t>OrderID</t>
+  </si>
+  <si>
+    <t>Ca Sản Xuất</t>
+  </si>
+  <si>
+    <t>Check</t>
   </si>
 </sst>
 </file>
@@ -164,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -187,9 +190,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -566,11 +566,11 @@
     <col min="7" max="7" width="30.140625" customWidth="1"/>
     <col min="8" max="8" width="19.140625" customWidth="1"/>
     <col min="9" max="9" width="17.85546875" customWidth="1"/>
-    <col min="10" max="10" width="13.140625" customWidth="1"/>
-    <col min="11" max="11" width="14.5703125" customWidth="1"/>
-    <col min="12" max="12" width="15.7109375" customWidth="1"/>
-    <col min="13" max="13" width="16.5703125" customWidth="1"/>
-    <col min="14" max="14" width="12.7109375" customWidth="1"/>
+    <col min="10" max="10" width="17.140625" customWidth="1"/>
+    <col min="11" max="11" width="21.5703125" customWidth="1"/>
+    <col min="12" max="12" width="23.42578125" customWidth="1"/>
+    <col min="13" max="13" width="24.85546875" customWidth="1"/>
+    <col min="14" max="14" width="20.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
@@ -618,7 +618,7 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
-      <c r="M3" s="11"/>
+      <c r="M3" s="10"/>
       <c r="N3" s="1"/>
     </row>
     <row r="4" spans="1:14" ht="73.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -630,7 +630,7 @@
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
@@ -644,42 +644,44 @@
         <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="D5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>4</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>5</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>0</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H5" s="8" t="s">
         <v>1</v>
       </c>
       <c r="I5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="J5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="K5" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="L5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="M5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="M5" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="N5" s="10"/>
+      <c r="N5" s="9" t="s">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
thêm cột excel chi tiết slab hrc2
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/HRC2_BBSL_PhoiTam.xlsx
+++ b/dataproduct.api/wwwroot/templates/HRC2_BBSL_PhoiTam.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\BIEUMAU_SANXUAT\Source\dataproduct.BE\dataproduct.api\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF4B3435-5DF9-4F20-95A9-D6ECF9639DD7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83DF01D8-8795-41AA-A90F-FBB10169CFC7}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="11805" xr2:uid="{8D26054B-D371-44B9-99F0-3A3B1380D846}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{8D26054B-D371-44B9-99F0-3A3B1380D846}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Máy đúc</t>
   </si>
@@ -67,6 +67,18 @@
   </si>
   <si>
     <t>OrderID</t>
+  </si>
+  <si>
+    <t>Ca BBSL</t>
+  </si>
+  <si>
+    <t>Chất lượng Gộp</t>
+  </si>
+  <si>
+    <t>Khối lượng phôi nguội</t>
+  </si>
+  <si>
+    <t>Khối lượng phôi nóng</t>
   </si>
 </sst>
 </file>
@@ -556,130 +568,160 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FE70C8B-98CB-4803-B542-3EE340B9292E}">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" customWidth="1"/>
-    <col min="3" max="4" width="19.140625" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" customWidth="1"/>
-    <col min="7" max="7" width="30.140625" customWidth="1"/>
-    <col min="8" max="8" width="19.140625" customWidth="1"/>
-    <col min="9" max="9" width="17.85546875" customWidth="1"/>
-    <col min="10" max="10" width="13.140625" customWidth="1"/>
-    <col min="11" max="11" width="14.5703125" customWidth="1"/>
-    <col min="12" max="12" width="15.7109375" customWidth="1"/>
-    <col min="13" max="13" width="16.5703125" customWidth="1"/>
-    <col min="14" max="14" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="3" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="7" width="19.140625" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" customWidth="1"/>
+    <col min="9" max="9" width="15.7109375" customWidth="1"/>
+    <col min="10" max="10" width="30.140625" customWidth="1"/>
+    <col min="11" max="11" width="19.140625" customWidth="1"/>
+    <col min="12" max="12" width="17.85546875" customWidth="1"/>
+    <col min="13" max="13" width="13.140625" customWidth="1"/>
+    <col min="14" max="14" width="23.5703125" customWidth="1"/>
+    <col min="15" max="15" width="14.5703125" customWidth="1"/>
+    <col min="16" max="16" width="15.7109375" customWidth="1"/>
+    <col min="17" max="17" width="16.5703125" customWidth="1"/>
+    <col min="18" max="18" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="2"/>
+      <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="H1" s="2"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
       <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="3"/>
+      <c r="R1" s="1"/>
     </row>
-    <row r="2" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="2"/>
+      <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="H2" s="2"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
       <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="1"/>
     </row>
-    <row r="3" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="2"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="H3" s="2"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
-      <c r="M3" s="11"/>
+      <c r="M3" s="1"/>
       <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="1"/>
     </row>
-    <row r="4" spans="1:14" ht="73.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="73.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
       <c r="D4" s="6"/>
-      <c r="E4" s="2"/>
+      <c r="E4" s="6"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
-      <c r="H4" s="7" t="s">
-        <v>12</v>
-      </c>
+      <c r="H4" s="2"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
+      <c r="K4" s="7" t="s">
+        <v>12</v>
+      </c>
       <c r="L4" s="6"/>
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
     </row>
-    <row r="5" spans="1:14" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="D5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="G5" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="I5" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="J5" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="K5" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="L5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="M5" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="N5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="O5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="P5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="M5" s="9" t="s">
+      <c r="Q5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="N5" s="10"/>
+      <c r="R5" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>